<commit_message>
docs(checklist): add Decision 0c topology row; mark Decisions 3 & 4 as spoke-only
Regenerated checklist.xlsx with new topology dropdown (spoke | standalone) and updated Decision 3 / 4a / 4b copy + Tab 3 tip to call out that standalone skips the hub decisions.
</commit_message>
<xml_diff>
--- a/config/checklist.xlsx
+++ b/config/checklist.xlsx
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A39"/>
+  <dimension ref="A1:A40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -561,176 +561,183 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">   - Pick a topology (row 0c) — 'spoke' if you already have an ALZ hub, 'standalone' for an isolated subscription. Standalone skips Decisions 3 and 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">   - Don't put GitHub tokens in the workbook. The wizard asks for them with hidden input.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr"/>
-    </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>2. Open 'Advanced Cluster Settings' only if you need to change cluster sizing, networking,</t>
-        </is>
-      </c>
+      <c r="A12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t>2. Open 'Advanced Cluster Settings' only if you need to change cluster sizing, networking,</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">   or upgrade behaviour. Most teams leave this tab alone.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr"/>
-    </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>3. Run the wizard and use the workbook as your reference:</t>
-        </is>
-      </c>
+      <c r="A15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">       Import-Module .\ALZ.AKS\ALZ.AKS.psd1 -Force</t>
+          <t>3. Run the wizard and use the workbook as your reference:</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">       Import-Module .\ALZ.AKS\ALZ.AKS.psd1 -Force</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">       Deploy-AKSLandingZone</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr"/>
-    </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>What the wizard does</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr"/>
-    </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Phase A — asks you the questions in this workbook and writes config files.</t>
-        </is>
-      </c>
+      <c r="A21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Phase B — creates the Azure resources, GitHub repos, runner, and pushes the Terraform code.</t>
+          <t>Phase A — asks you the questions in this workbook and writes config files.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
+          <t>Phase B — creates the Azure resources, GitHub repos, runner, and pushes the Terraform code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
           <t>Phase C — your PRs in the new GitHub repo run plan/apply and deploy the cluster.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr"/>
-    </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>GitHub tokens — scopes you need</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr"/>
-    </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Main token (always):    repo, workflow, admin:org (Members Read &amp; Write)</t>
-        </is>
-      </c>
+      <c r="A27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t>Main token (always):    repo, workflow, admin:org (Members Read &amp; Write)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
           <t>Runner token (if 9a is true):  admin:org (full)</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr"/>
-    </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>Resource names you will see</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr"/>
-    </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Pattern: {service}-{env}-{region-short}-{number}</t>
-        </is>
-      </c>
+      <c r="A32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Example with defaults (aksapplz, prod, swedencentral, 1):</t>
+          <t>Pattern: {service}-{env}-{region-short}-{number}</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Resource group for state:     rg-aksapplz-prod-sc-001</t>
+          <t>Example with defaults (aksapplz, prod, swedencentral, 1):</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Resource group for identity:  rg-aksapplz-prod-sc-identity</t>
+          <t xml:space="preserve">  Resource group for state:     rg-aksapplz-prod-sc-001</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Resource group for runner:    rg-aksapplz-prod-sc-agents     (only with self-hosted runners)</t>
+          <t xml:space="preserve">  Resource group for identity:  rg-aksapplz-prod-sc-identity</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  GitHub repository:            aksapplz-prod</t>
+          <t xml:space="preserve">  Resource group for runner:    rg-aksapplz-prod-sc-agents     (only with self-hosted runners)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  GitHub templates repo:        aksapplz-prod-templates</t>
+          <t xml:space="preserve">  GitHub repository:            aksapplz-prod</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  GitHub templates repo:        aksapplz-prod-templates</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  Approver team:                aksapplz-prod-approvers</t>
         </is>
@@ -747,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -872,226 +879,227 @@
       <c r="F7" s="10" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr"/>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>0c</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>topology</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>How the AKS landing zone connects to the network. 'spoke' peers to an existing ALZ hub and routes egress through the hub firewall; 'standalone' has no hub, no peering, and uses a NAT gateway for egress (Decisions 3 and 4 are ignored).</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>spoke      (default; peer to existing ALZ hub)
+standalone (no hub, NAT egress only)</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>spoke</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr"/>
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>WHERE TO DEPLOY</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="7" t="n"/>
-      <c r="F8" s="7" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>bootstrap_location</t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>Main Azure region for the cluster and supporting resources.</t>
-        </is>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>swedencentral, westeurope, eastus2 ...</t>
-        </is>
-      </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>swedencentral</t>
-        </is>
-      </c>
-      <c r="F9" s="10" t="inlineStr"/>
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="7" t="n"/>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>bootstrap_location</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Main Azure region for the cluster and supporting resources.</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>swedencentral, westeurope, eastus2 ...</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>swedencentral</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>aks_landing_zone_subscription_id</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>Subscription where the AKS cluster will be created.</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>Subscription ID (GUID).
 Leave blank to use whatever `az` is logged into.</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="E11" s="9" t="inlineStr">
         <is>
           <t>(current az subscription)</t>
         </is>
       </c>
-      <c r="F10" s="10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="F11" s="10" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>connectivity_subscription_id</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>Subscription that holds your existing hub network (firewall, VPN).</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Subscription that holds your existing hub network (firewall, VPN). Only required when topology = spoke; leave blank for standalone.</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>Subscription ID (GUID).</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr"/>
-      <c r="F11" s="10" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr"/>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>HUB NETWORK (you already have this)</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="n"/>
-      <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
-      <c r="F12" s="7" t="n"/>
+      <c r="E12" s="9" t="inlineStr"/>
+      <c r="F12" s="10" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>4a</t>
-        </is>
-      </c>
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>hub_vnet_resource_id</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>Full ID of your hub VNet. The wizard lists hubs found in Decision 3 and fills this in.</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="inlineStr">
-        <is>
-          <t>/subscriptions/&lt;id&gt;/resourceGroups/&lt;rg&gt;/providers/Microsoft.Network/virtualNetworks/&lt;name&gt;</t>
-        </is>
-      </c>
-      <c r="E13" s="9" t="inlineStr"/>
-      <c r="F13" s="10" t="inlineStr"/>
+      <c r="A13" s="7" t="inlineStr"/>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>HUB NETWORK (only when topology = spoke)</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
+          <t>4a</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>hub_vnet_resource_id</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Full ID of your hub VNet. The wizard lists hubs found in Decision 3 and fills this in. Leave blank when topology = standalone.</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>/subscriptions/&lt;id&gt;/resourceGroups/&lt;rg&gt;/providers/Microsoft.Network/virtualNetworks/&lt;name&gt;</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr"/>
+      <c r="F14" s="10" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
           <t>4b</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>hub_firewall_private_ip</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>Private IP of your hub firewall. Traffic leaving the cluster routes through this.</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Private IP of your hub firewall. Traffic leaving the cluster routes through this. Leave blank when topology = standalone.</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>10.0.0.4</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="E15" s="9" t="inlineStr">
         <is>
           <t>10.0.0.4</t>
         </is>
       </c>
-      <c r="F14" s="10" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr"/>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="F15" s="10" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr"/>
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>SPOKE NETWORK (the new VNet for AKS)</t>
         </is>
       </c>
-      <c r="C15" s="7" t="n"/>
-      <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
-      <c r="F15" s="7" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>5a</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>spoke_vnet_address_space</t>
-        </is>
-      </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>Address range for the new spoke VNet. Must not overlap with any other VNet.</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>10.10.0.0/16</t>
-        </is>
-      </c>
-      <c r="E16" s="9" t="inlineStr">
-        <is>
-          <t>10.10.0.0/16</t>
-        </is>
-      </c>
-      <c r="F16" s="10" t="inlineStr"/>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="7" t="n"/>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>5b</t>
+          <t>5a</t>
         </is>
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>subnet_address_prefix_aks_system_nodes</t>
+          <t>spoke_vnet_address_space</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>Small subnet for the system node pool (runs cluster add-ons only).</t>
+          <t>Address range for the new spoke VNet. Must not overlap with any other VNet.</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>10.10.0.0/24  (256 addresses)</t>
+          <t>10.10.0.0/16</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>10.10.0.0/24</t>
+          <t>10.10.0.0/16</t>
         </is>
       </c>
       <c r="F17" s="10" t="inlineStr"/>
@@ -1099,27 +1107,27 @@
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>5c</t>
+          <t>5b</t>
         </is>
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>subnet_address_prefix_aks_user_nodes</t>
+          <t>subnet_address_prefix_aks_system_nodes</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>Bigger subnet for your application workloads.</t>
+          <t>Small subnet for the system node pool (runs cluster add-ons only).</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>10.10.16.0/22  (1024 addresses)</t>
+          <t>10.10.0.0/24  (256 addresses)</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>10.10.16.0/22</t>
+          <t>10.10.0.0/24</t>
         </is>
       </c>
       <c r="F18" s="10" t="inlineStr"/>
@@ -1127,27 +1135,27 @@
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>5d</t>
+          <t>5c</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>subnet_address_prefix_aks_api_server</t>
+          <t>subnet_address_prefix_aks_user_nodes</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>Subnet for the private Kubernetes API server.</t>
+          <t>Bigger subnet for your application workloads.</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>10.10.20.0/28  (Azure requires at least /28)</t>
+          <t>10.10.16.0/22  (1024 addresses)</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>10.10.20.0/28</t>
+          <t>10.10.16.0/22</t>
         </is>
       </c>
       <c r="F19" s="10" t="inlineStr"/>
@@ -1155,27 +1163,27 @@
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>5e</t>
+          <t>5d</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>subnet_address_prefix_app_gateway</t>
+          <t>subnet_address_prefix_aks_api_server</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>Subnet for Application Gateway (web traffic in).</t>
+          <t>Subnet for the private Kubernetes API server.</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>10.10.21.0/24</t>
+          <t>10.10.20.0/28  (Azure requires at least /28)</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>10.10.21.0/24</t>
+          <t>10.10.20.0/28</t>
         </is>
       </c>
       <c r="F20" s="10" t="inlineStr"/>
@@ -1183,27 +1191,27 @@
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>5f</t>
+          <t>5e</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>subnet_address_prefix_private_endpoints</t>
+          <t>subnet_address_prefix_app_gateway</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>Subnet for private endpoints (ACR, Key Vault, storage).</t>
+          <t>Subnet for Application Gateway (web traffic in).</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>10.10.22.0/24</t>
+          <t>10.10.21.0/24</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>10.10.22.0/24</t>
+          <t>10.10.21.0/24</t>
         </is>
       </c>
       <c r="F21" s="10" t="inlineStr"/>
@@ -1211,95 +1219,95 @@
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
+          <t>5f</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>subnet_address_prefix_private_endpoints</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Subnet for private endpoints (ACR, Key Vault, storage).</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>10.10.22.0/24</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>10.10.22.0/24</t>
+        </is>
+      </c>
+      <c r="F22" s="10" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
           <t>5g</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>subnet_address_prefix_ingress</t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr">
+      <c r="C23" s="9" t="inlineStr">
         <is>
           <t>Subnet for the internal load balancer that fronts your apps.</t>
         </is>
       </c>
-      <c r="D22" s="9" t="inlineStr">
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t>10.10.23.0/24</t>
         </is>
       </c>
-      <c r="E22" s="9" t="inlineStr">
+      <c r="E23" s="9" t="inlineStr">
         <is>
           <t>10.10.23.0/24</t>
         </is>
       </c>
-      <c r="F22" s="10" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="7" t="inlineStr"/>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="F23" s="10" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr"/>
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>CLUSTER SETTINGS</t>
         </is>
       </c>
-      <c r="C23" s="7" t="n"/>
-      <c r="D23" s="7" t="n"/>
-      <c r="E23" s="7" t="n"/>
-      <c r="F23" s="7" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="8" t="inlineStr">
-        <is>
-          <t>6a</t>
-        </is>
-      </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>kubernetes_version</t>
-        </is>
-      </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>Kubernetes version. The wizard lists the latest versions available in your region — usually just pick the top one.</t>
-        </is>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>Example: 1.33.6</t>
-        </is>
-      </c>
-      <c r="E24" s="9" t="inlineStr">
-        <is>
-          <t>(latest in region)</t>
-        </is>
-      </c>
-      <c r="F24" s="10" t="inlineStr"/>
+      <c r="C24" s="7" t="n"/>
+      <c r="D24" s="7" t="n"/>
+      <c r="E24" s="7" t="n"/>
+      <c r="F24" s="7" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>6b</t>
+          <t>6a</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>aks_sku_tier</t>
+          <t>kubernetes_version</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>Cluster pricing tier. Standard is fine for most clusters; Premium adds long-term support and is required for regulated scenarios.</t>
+          <t>Kubernetes version. The wizard lists the latest versions available in your region — usually just pick the top one.</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>Free | Standard | Premium</t>
+          <t>Example: 1.33.6</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>(latest in region)</t>
         </is>
       </c>
       <c r="F25" s="10" t="inlineStr"/>
@@ -1307,164 +1315,164 @@
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
+          <t>6b</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>aks_sku_tier</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Cluster pricing tier. Standard is fine for most clusters; Premium adds long-term support and is required for regulated scenarios.</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>Free | Standard | Premium</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
           <t>6c</t>
         </is>
       </c>
-      <c r="B26" s="9" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t>aks_private_cluster</t>
         </is>
       </c>
-      <c r="C26" s="9" t="inlineStr">
+      <c r="C27" s="9" t="inlineStr">
         <is>
           <t>Hide the Kubernetes API behind your private network (no public endpoint).</t>
         </is>
       </c>
-      <c r="D26" s="9" t="inlineStr">
+      <c r="D27" s="9" t="inlineStr">
         <is>
           <t>true  (recommended)
 false (only for internet-facing demos)</t>
         </is>
       </c>
-      <c r="E26" s="9" t="inlineStr">
+      <c r="E27" s="9" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="F26" s="10" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="8" t="inlineStr">
+      <c r="F27" s="10" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t>6d</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>aks_admin_group_object_ids</t>
         </is>
       </c>
-      <c r="C27" s="9" t="inlineStr">
+      <c r="C28" s="9" t="inlineStr">
         <is>
           <t>Entra ID group(s) whose members can manage the cluster. Create the group in Entra ID first and paste the object ID.</t>
         </is>
       </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="D28" s="9" t="inlineStr">
         <is>
           <t>["00000000-0000-0000-0000-000000000000"]</t>
         </is>
       </c>
-      <c r="E27" s="9" t="inlineStr">
+      <c r="E28" s="9" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="F27" s="10" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="7" t="inlineStr"/>
-      <c r="B28" s="7" t="inlineStr">
+      <c r="F28" s="10" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr"/>
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>WHERE STATE LIVES</t>
         </is>
       </c>
-      <c r="C28" s="7" t="n"/>
-      <c r="D28" s="7" t="n"/>
-      <c r="E28" s="7" t="n"/>
-      <c r="F28" s="7" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="8" t="inlineStr">
+      <c r="C29" s="7" t="n"/>
+      <c r="D29" s="7" t="n"/>
+      <c r="E29" s="7" t="n"/>
+      <c r="F29" s="7" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>bootstrap_subscription_id</t>
         </is>
       </c>
-      <c r="C29" s="9" t="inlineStr">
+      <c r="C30" s="9" t="inlineStr">
         <is>
           <t>Subscription that holds the Terraform state storage and the runner. Usually the same as Decision 2.</t>
         </is>
       </c>
-      <c r="D29" s="9" t="inlineStr">
+      <c r="D30" s="9" t="inlineStr">
         <is>
           <t>Subscription ID (GUID), or leave blank.</t>
         </is>
       </c>
-      <c r="E29" s="9" t="inlineStr">
+      <c r="E30" s="9" t="inlineStr">
         <is>
           <t>(same as Decision 2)</t>
         </is>
       </c>
-      <c r="F29" s="10" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="7" t="inlineStr"/>
-      <c r="B30" s="7" t="inlineStr">
+      <c r="F30" s="10" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr"/>
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>NAMING</t>
         </is>
       </c>
-      <c r="C30" s="7" t="n"/>
-      <c r="D30" s="7" t="n"/>
-      <c r="E30" s="7" t="n"/>
-      <c r="F30" s="7" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
-        <is>
-          <t>8a</t>
-        </is>
-      </c>
-      <c r="B31" s="9" t="inlineStr">
-        <is>
-          <t>service_name</t>
-        </is>
-      </c>
-      <c r="C31" s="9" t="inlineStr">
-        <is>
-          <t>Short name of your workload. Used in every resource name.</t>
-        </is>
-      </c>
-      <c r="D31" s="9" t="inlineStr">
-        <is>
-          <t>aksapplz, payments, shop</t>
-        </is>
-      </c>
-      <c r="E31" s="9" t="inlineStr">
-        <is>
-          <t>aksapplz</t>
-        </is>
-      </c>
-      <c r="F31" s="10" t="inlineStr"/>
+      <c r="C31" s="7" t="n"/>
+      <c r="D31" s="7" t="n"/>
+      <c r="E31" s="7" t="n"/>
+      <c r="F31" s="7" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t>8b</t>
+          <t>8a</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>environment_name</t>
+          <t>service_name</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>Environment label. Used in every resource name.</t>
+          <t>Short name of your workload. Used in every resource name.</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>prod, dev, test</t>
+          <t>aksapplz, payments, shop</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>prod</t>
+          <t>aksapplz</t>
         </is>
       </c>
       <c r="F32" s="10" t="inlineStr"/>
@@ -1472,160 +1480,160 @@
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
+          <t>8b</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>environment_name</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>Environment label. Used in every resource name.</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>prod, dev, test</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t>prod</t>
+        </is>
+      </c>
+      <c r="F33" s="10" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
           <t>8c</t>
         </is>
       </c>
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B34" s="9" t="inlineStr">
         <is>
           <t>postfix_number</t>
         </is>
       </c>
-      <c r="C33" s="9" t="inlineStr">
+      <c r="C34" s="9" t="inlineStr">
         <is>
           <t>Number that makes resource names unique. Bump this if you redeploy.</t>
         </is>
       </c>
-      <c r="D33" s="9" t="inlineStr">
+      <c r="D34" s="9" t="inlineStr">
         <is>
           <t>1, 2, 3 ...</t>
         </is>
       </c>
-      <c r="E33" s="9" t="inlineStr">
+      <c r="E34" s="9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="F33" s="10" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="7" t="inlineStr"/>
-      <c r="B34" s="7" t="inlineStr">
+      <c r="F34" s="10" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr"/>
+      <c r="B35" s="7" t="inlineStr">
         <is>
           <t>RUNNERS</t>
         </is>
       </c>
-      <c r="C34" s="7" t="n"/>
-      <c r="D34" s="7" t="n"/>
-      <c r="E34" s="7" t="n"/>
-      <c r="F34" s="7" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
+      <c r="C35" s="7" t="n"/>
+      <c r="D35" s="7" t="n"/>
+      <c r="E35" s="7" t="n"/>
+      <c r="F35" s="7" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>9a</t>
         </is>
       </c>
-      <c r="B35" s="9" t="inlineStr">
+      <c r="B36" s="9" t="inlineStr">
         <is>
           <t>use_self_hosted_runners</t>
         </is>
       </c>
-      <c r="C35" s="9" t="inlineStr">
+      <c r="C36" s="9" t="inlineStr">
         <is>
           <t>Run GitHub Actions on a small container inside Azure (needed for private clusters so CI/CD can reach the API).</t>
         </is>
       </c>
-      <c r="D35" s="9" t="inlineStr">
+      <c r="D36" s="9" t="inlineStr">
         <is>
           <t>true  (required for private clusters)
 false (use GitHub-hosted runners)</t>
         </is>
       </c>
-      <c r="E35" s="9" t="inlineStr">
+      <c r="E36" s="9" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="F35" s="10" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
+      <c r="F36" s="10" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
         <is>
           <t>9b</t>
         </is>
       </c>
-      <c r="B36" s="9" t="inlineStr">
+      <c r="B37" s="9" t="inlineStr">
         <is>
           <t>use_private_networking</t>
         </is>
       </c>
-      <c r="C36" s="9" t="inlineStr">
+      <c r="C37" s="9" t="inlineStr">
         <is>
           <t>Put the runner and Container Registry on a private network. Recommended.</t>
         </is>
       </c>
-      <c r="D36" s="9" t="inlineStr">
+      <c r="D37" s="9" t="inlineStr">
         <is>
           <t>true  (recommended)
 false (public networking, ACR Basic)</t>
         </is>
       </c>
-      <c r="E36" s="9" t="inlineStr">
+      <c r="E37" s="9" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="F36" s="10" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="7" t="inlineStr"/>
-      <c r="B37" s="7" t="inlineStr">
+      <c r="F37" s="10" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr"/>
+      <c r="B38" s="7" t="inlineStr">
         <is>
           <t>GITHUB</t>
         </is>
       </c>
-      <c r="C37" s="7" t="n"/>
-      <c r="D37" s="7" t="n"/>
-      <c r="E37" s="7" t="n"/>
-      <c r="F37" s="7" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="8" t="inlineStr">
-        <is>
-          <t>10a</t>
-        </is>
-      </c>
-      <c r="B38" s="9" t="inlineStr">
-        <is>
-          <t>github_personal_access_token</t>
-        </is>
-      </c>
-      <c r="C38" s="9" t="inlineStr">
-        <is>
-          <t>GitHub token used to create the repos. You will be prompted (input is hidden); you do NOT need to put it here.</t>
-        </is>
-      </c>
-      <c r="D38" s="9" t="inlineStr">
-        <is>
-          <t>Scopes needed: repo, workflow, admin:org (Read &amp; Write members).</t>
-        </is>
-      </c>
-      <c r="E38" s="9" t="inlineStr">
-        <is>
-          <t>(prompted in wizard)</t>
-        </is>
-      </c>
-      <c r="F38" s="10" t="inlineStr"/>
+      <c r="C38" s="7" t="n"/>
+      <c r="D38" s="7" t="n"/>
+      <c r="E38" s="7" t="n"/>
+      <c r="F38" s="7" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>10b</t>
+          <t>10a</t>
         </is>
       </c>
       <c r="B39" s="9" t="inlineStr">
         <is>
-          <t>github_runners_personal_access_token</t>
+          <t>github_personal_access_token</t>
         </is>
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>Second token used to register the self-hosted runner. Also prompted; only asked when 9a is true.</t>
+          <t>GitHub token used to create the repos. You will be prompted (input is hidden); you do NOT need to put it here.</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>Scope needed: admin:org (full).</t>
+          <t>Scopes needed: repo, workflow, admin:org (Read &amp; Write members).</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr">
@@ -1638,109 +1646,109 @@
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
-          <t>10c</t>
+          <t>10b</t>
         </is>
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>github_organization_name</t>
+          <t>github_runners_personal_access_token</t>
         </is>
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>GitHub organisation name where the two repos will be created.</t>
+          <t>Second token used to register the self-hosted runner. Also prompted; only asked when 9a is true.</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>contoso</t>
-        </is>
-      </c>
-      <c r="E40" s="9" t="inlineStr"/>
+          <t>Scope needed: admin:org (full).</t>
+        </is>
+      </c>
+      <c r="E40" s="9" t="inlineStr">
+        <is>
+          <t>(prompted in wizard)</t>
+        </is>
+      </c>
       <c r="F40" s="10" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
+          <t>10c</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>github_organization_name</t>
+        </is>
+      </c>
+      <c r="C41" s="9" t="inlineStr">
+        <is>
+          <t>GitHub organisation name where the two repos will be created.</t>
+        </is>
+      </c>
+      <c r="D41" s="9" t="inlineStr">
+        <is>
+          <t>contoso</t>
+        </is>
+      </c>
+      <c r="E41" s="9" t="inlineStr"/>
+      <c r="F41" s="10" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
           <t>10d</t>
         </is>
       </c>
-      <c r="B41" s="9" t="inlineStr">
+      <c r="B42" s="9" t="inlineStr">
         <is>
           <t>apply_approvers</t>
         </is>
       </c>
-      <c r="C41" s="9" t="inlineStr">
+      <c r="C42" s="9" t="inlineStr">
         <is>
           <t>GitHub usernames who must approve before a deployment goes live.</t>
         </is>
       </c>
-      <c r="D41" s="9" t="inlineStr">
+      <c r="D42" s="9" t="inlineStr">
         <is>
           <t>["alice", "bob"]</t>
         </is>
       </c>
-      <c r="E41" s="9" t="inlineStr">
+      <c r="E42" s="9" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="F41" s="10" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="7" t="inlineStr"/>
-      <c r="B42" s="7" t="inlineStr">
+      <c r="F42" s="10" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="inlineStr"/>
+      <c r="B43" s="7" t="inlineStr">
         <is>
           <t>ADD-ONS (turn things on or off)</t>
         </is>
       </c>
-      <c r="C42" s="7" t="n"/>
-      <c r="D42" s="7" t="n"/>
-      <c r="E42" s="7" t="n"/>
-      <c r="F42" s="7" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="inlineStr">
-        <is>
-          <t>11a</t>
-        </is>
-      </c>
-      <c r="B43" s="9" t="inlineStr">
-        <is>
-          <t>enable_defender</t>
-        </is>
-      </c>
-      <c r="C43" s="9" t="inlineStr">
-        <is>
-          <t>Scans the cluster for security threats in real time.</t>
-        </is>
-      </c>
-      <c r="D43" s="9" t="inlineStr">
-        <is>
-          <t>true | false</t>
-        </is>
-      </c>
-      <c r="E43" s="9" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="F43" s="10" t="inlineStr"/>
+      <c r="C43" s="7" t="n"/>
+      <c r="D43" s="7" t="n"/>
+      <c r="E43" s="7" t="n"/>
+      <c r="F43" s="7" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="8" t="inlineStr">
         <is>
-          <t>11b</t>
+          <t>11a</t>
         </is>
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>enable_workload_identity</t>
+          <t>enable_defender</t>
         </is>
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>Lets pods talk to Azure services without passwords.</t>
+          <t>Scans the cluster for security threats in real time.</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
@@ -1758,17 +1766,17 @@
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>11c</t>
+          <t>11b</t>
         </is>
       </c>
       <c r="B45" s="9" t="inlineStr">
         <is>
-          <t>enable_azure_policy</t>
+          <t>enable_workload_identity</t>
         </is>
       </c>
       <c r="C45" s="9" t="inlineStr">
         <is>
-          <t>Enforces rules in the cluster (e.g. block containers running as root).</t>
+          <t>Lets pods talk to Azure services without passwords.</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
@@ -1786,17 +1794,17 @@
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
         <is>
-          <t>11d</t>
+          <t>11c</t>
         </is>
       </c>
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>enable_prometheus</t>
+          <t>enable_azure_policy</t>
         </is>
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>Collects cluster metrics.</t>
+          <t>Enforces rules in the cluster (e.g. block containers running as root).</t>
         </is>
       </c>
       <c r="D46" s="9" t="inlineStr">
@@ -1814,17 +1822,17 @@
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>11e</t>
+          <t>11d</t>
         </is>
       </c>
       <c r="B47" s="9" t="inlineStr">
         <is>
-          <t>enable_grafana</t>
+          <t>enable_prometheus</t>
         </is>
       </c>
       <c r="C47" s="9" t="inlineStr">
         <is>
-          <t>Dashboards for the metrics above.</t>
+          <t>Collects cluster metrics.</t>
         </is>
       </c>
       <c r="D47" s="9" t="inlineStr">
@@ -1842,17 +1850,17 @@
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
         <is>
-          <t>11f</t>
+          <t>11e</t>
         </is>
       </c>
       <c r="B48" s="9" t="inlineStr">
         <is>
-          <t>enable_app_gateway</t>
+          <t>enable_grafana</t>
         </is>
       </c>
       <c r="C48" s="9" t="inlineStr">
         <is>
-          <t>Application Gateway with a Web Application Firewall in front of the cluster.</t>
+          <t>Dashboards for the metrics above.</t>
         </is>
       </c>
       <c r="D48" s="9" t="inlineStr">
@@ -1870,17 +1878,17 @@
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t>11g</t>
+          <t>11f</t>
         </is>
       </c>
       <c r="B49" s="9" t="inlineStr">
         <is>
-          <t>enable_keda</t>
+          <t>enable_app_gateway</t>
         </is>
       </c>
       <c r="C49" s="9" t="inlineStr">
         <is>
-          <t>Auto-scales pods based on events (queue length, HTTP requests, etc.).</t>
+          <t>Application Gateway with a Web Application Firewall in front of the cluster.</t>
         </is>
       </c>
       <c r="D49" s="9" t="inlineStr">
@@ -1898,17 +1906,17 @@
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
         <is>
-          <t>11h</t>
+          <t>11g</t>
         </is>
       </c>
       <c r="B50" s="9" t="inlineStr">
         <is>
-          <t>enable_vpa</t>
+          <t>enable_keda</t>
         </is>
       </c>
       <c r="C50" s="9" t="inlineStr">
         <is>
-          <t>Auto-adjusts CPU and memory requests for pods.</t>
+          <t>Auto-scales pods based on events (queue length, HTTP requests, etc.).</t>
         </is>
       </c>
       <c r="D50" s="9" t="inlineStr">
@@ -1918,7 +1926,7 @@
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>false  (true for regulated / multi-region)</t>
+          <t>true</t>
         </is>
       </c>
       <c r="F50" s="10" t="inlineStr"/>
@@ -1926,17 +1934,17 @@
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>11i</t>
+          <t>11h</t>
         </is>
       </c>
       <c r="B51" s="9" t="inlineStr">
         <is>
-          <t>enable_node_auto_provisioning</t>
+          <t>enable_vpa</t>
         </is>
       </c>
       <c r="C51" s="9" t="inlineStr">
         <is>
-          <t>Cluster creates new node sizes on demand instead of using fixed pools.</t>
+          <t>Auto-adjusts CPU and memory requests for pods.</t>
         </is>
       </c>
       <c r="D51" s="9" t="inlineStr">
@@ -1946,7 +1954,7 @@
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>false  (true for multi-region)</t>
+          <t>false  (true for regulated / multi-region)</t>
         </is>
       </c>
       <c r="F51" s="10" t="inlineStr"/>
@@ -1954,17 +1962,17 @@
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
         <is>
-          <t>11j</t>
+          <t>11i</t>
         </is>
       </c>
       <c r="B52" s="9" t="inlineStr">
         <is>
-          <t>enable_istio</t>
+          <t>enable_node_auto_provisioning</t>
         </is>
       </c>
       <c r="C52" s="9" t="inlineStr">
         <is>
-          <t>Service mesh with mTLS between pods. Needed for some compliance standards.</t>
+          <t>Cluster creates new node sizes on demand instead of using fixed pools.</t>
         </is>
       </c>
       <c r="D52" s="9" t="inlineStr">
@@ -1974,7 +1982,7 @@
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>false  (true for regulated)</t>
+          <t>false  (true for multi-region)</t>
         </is>
       </c>
       <c r="F52" s="10" t="inlineStr"/>
@@ -1982,17 +1990,17 @@
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t>11k</t>
+          <t>11j</t>
         </is>
       </c>
       <c r="B53" s="9" t="inlineStr">
         <is>
-          <t>enable_flux</t>
+          <t>enable_istio</t>
         </is>
       </c>
       <c r="C53" s="9" t="inlineStr">
         <is>
-          <t>GitOps — the cluster pulls its configuration from a Git repo.</t>
+          <t>Service mesh with mTLS between pods. Needed for some compliance standards.</t>
         </is>
       </c>
       <c r="D53" s="9" t="inlineStr">
@@ -2002,7 +2010,7 @@
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>false  (true for multi-region)</t>
+          <t>false  (true for regulated)</t>
         </is>
       </c>
       <c r="F53" s="10" t="inlineStr"/>
@@ -2010,17 +2018,17 @@
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t>11l</t>
+          <t>11k</t>
         </is>
       </c>
       <c r="B54" s="9" t="inlineStr">
         <is>
-          <t>enable_dapr</t>
+          <t>enable_flux</t>
         </is>
       </c>
       <c r="C54" s="9" t="inlineStr">
         <is>
-          <t>Building blocks for microservices (pub/sub, state, secrets).</t>
+          <t>GitOps — the cluster pulls its configuration from a Git repo.</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
@@ -2030,7 +2038,7 @@
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>false  (true for multi-region)</t>
         </is>
       </c>
       <c r="F54" s="10" t="inlineStr"/>
@@ -2038,17 +2046,17 @@
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t>11m</t>
+          <t>11l</t>
         </is>
       </c>
       <c r="B55" s="9" t="inlineStr">
         <is>
-          <t>enable_fips</t>
+          <t>enable_dapr</t>
         </is>
       </c>
       <c r="C55" s="9" t="inlineStr">
         <is>
-          <t>Use FIPS 140-2 compliant node OS (US Federal / PCI).</t>
+          <t>Building blocks for microservices (pub/sub, state, secrets).</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
@@ -2058,7 +2066,7 @@
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>false  (true for regulated)</t>
+          <t>false</t>
         </is>
       </c>
       <c r="F55" s="10" t="inlineStr"/>
@@ -2066,17 +2074,17 @@
     <row r="56">
       <c r="A56" s="8" t="inlineStr">
         <is>
-          <t>11n</t>
+          <t>11m</t>
         </is>
       </c>
       <c r="B56" s="9" t="inlineStr">
         <is>
-          <t>enable_backup</t>
+          <t>enable_fips</t>
         </is>
       </c>
       <c r="C56" s="9" t="inlineStr">
         <is>
-          <t>Azure Backup for cluster resources and persistent volumes.</t>
+          <t>Use FIPS 140-2 compliant node OS (US Federal / PCI).</t>
         </is>
       </c>
       <c r="D56" s="9" t="inlineStr">
@@ -2086,7 +2094,7 @@
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>false  (true for regulated / multi-region)</t>
+          <t>false  (true for regulated)</t>
         </is>
       </c>
       <c r="F56" s="10" t="inlineStr"/>
@@ -2094,63 +2102,91 @@
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
+          <t>11n</t>
+        </is>
+      </c>
+      <c r="B57" s="9" t="inlineStr">
+        <is>
+          <t>enable_backup</t>
+        </is>
+      </c>
+      <c r="C57" s="9" t="inlineStr">
+        <is>
+          <t>Azure Backup for cluster resources and persistent volumes.</t>
+        </is>
+      </c>
+      <c r="D57" s="9" t="inlineStr">
+        <is>
+          <t>true | false</t>
+        </is>
+      </c>
+      <c r="E57" s="9" t="inlineStr">
+        <is>
+          <t>false  (true for regulated / multi-region)</t>
+        </is>
+      </c>
+      <c r="F57" s="10" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
+        <is>
           <t>11o</t>
         </is>
       </c>
-      <c r="B57" s="9" t="inlineStr">
+      <c r="B58" s="9" t="inlineStr">
         <is>
           <t>enable_cost_analysis</t>
         </is>
       </c>
-      <c r="C57" s="9" t="inlineStr">
+      <c r="C58" s="9" t="inlineStr">
         <is>
           <t>Cost breakdown per namespace in the Azure portal.</t>
         </is>
       </c>
-      <c r="D57" s="9" t="inlineStr">
+      <c r="D58" s="9" t="inlineStr">
         <is>
           <t>true | false</t>
         </is>
       </c>
-      <c r="E57" s="9" t="inlineStr">
+      <c r="E58" s="9" t="inlineStr">
         <is>
           <t>false  (true for regulated)</t>
         </is>
       </c>
-      <c r="F57" s="10" t="inlineStr"/>
+      <c r="F58" s="10" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B30:F30"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B34:F34"/>
-    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="B24:F24"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B38:F38"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="B42:F42"/>
     <mergeCell ref="B5:F5"/>
-    <mergeCell ref="B37:F37"/>
-    <mergeCell ref="B23:F23"/>
-    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B35:F35"/>
   </mergeCells>
-  <dataValidations count="20">
+  <dataValidations count="21">
     <dataValidation sqref="F6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"single_region_baseline,multi_region_baseline,single_region_regulated,multi_region_regulated"</formula1>
     </dataValidation>
-    <dataValidation sqref="F25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"spoke,standalone"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Free,Standard,Premium"</formula1>
     </dataValidation>
-    <dataValidation sqref="F26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"true,false"</formula1>
-    </dataValidation>
-    <dataValidation sqref="F35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"true,false"</formula1>
     </dataValidation>
     <dataValidation sqref="F36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"true,false"</formula1>
     </dataValidation>
-    <dataValidation sqref="F43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"true,false"</formula1>
     </dataValidation>
     <dataValidation sqref="F44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -2195,6 +2231,9 @@
     <dataValidation sqref="F57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"true,false"</formula1>
     </dataValidation>
+    <dataValidation sqref="F58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"true,false"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
checklist: add Reference (Microsoft Learn) and Comments columns; home: 4-step journey (plan first)
Add a clickable Microsoft Learn / GitHub Docs reference link and a free-form Comments column to both checklist tabs (driven by a REFERENCES lookup). Restructure the home-page journey from 3 to 4 steps so decisions come first: Plan -> Choose a scenario -> Prepare -> Deploy.
</commit_message>
<xml_diff>
--- a/config/checklist.xlsx
+++ b/config/checklist.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -54,6 +54,12 @@
     <font>
       <name val="Segoe UI"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="5">
@@ -108,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -134,6 +140,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -501,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A40"/>
+  <dimension ref="A1:A42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -561,65 +570,69 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Pick a topology (row 0c) — 'spoke' if you already have an ALZ hub, 'hub_and_spoke' to create a new hub this run, or 'standalone' for an isolated subscription. Standalone skips Decisions 3 and 4.</t>
+          <t xml:space="preserve">   - Use the 'Reference' column links to read the Microsoft Learn docs for any setting.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Don't put GitHub tokens in the workbook. The wizard asks for them with hidden input.</t>
+          <t xml:space="preserve">   - Use the 'Comments' column (yellow) to record why you chose a value — handy for your team and auditors.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr"/>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Pick a topology (row 0c) — 'spoke' if you already have an ALZ hub, 'hub_and_spoke' to create a new hub this run, or 'standalone' for an isolated subscription. Standalone skips Decisions 3 and 4.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">   - Don't put GitHub tokens in the workbook. The wizard asks for them with hidden input.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t>2. Open 'Advanced Cluster Settings' only if you need to change cluster sizing, networking,</t>
         </is>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   or upgrade behaviour. Most teams leave this tab alone.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>3. Run the wizard and use the workbook as your reference:</t>
+          <t xml:space="preserve">   or upgrade behaviour. Most teams leave this tab alone.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       Import-Module .\ALZ.AKS\ALZ.AKS.psd1 -Force</t>
-        </is>
-      </c>
+      <c r="A17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>3. Run the wizard and use the workbook as your reference:</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">       Import-Module .\ALZ.AKS\ALZ.AKS.psd1 -Force</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">       Deploy-AKSLandingZone</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>What the wizard does</t>
         </is>
       </c>
     </row>
@@ -627,33 +640,33 @@
       <c r="A21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Phase A — asks you the questions in this workbook and writes config files.</t>
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>What the wizard does</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Phase B — creates the Azure resources, GitHub repos, runner, and pushes the Terraform code.</t>
-        </is>
-      </c>
+      <c r="A23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
+          <t>Phase A — asks you the questions in this workbook and writes config files.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Phase B — creates the Azure resources, GitHub repos, runner, and pushes the Terraform code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
           <t>Phase C — your PRs in the new GitHub repo run plan/apply and deploy the cluster.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>GitHub tokens — scopes you need</t>
         </is>
       </c>
     </row>
@@ -661,26 +674,26 @@
       <c r="A27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>GitHub tokens — scopes you need</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>Main token (always):    repo, workflow, admin:org (Members Read &amp; Write)</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>Runner token (if 9a is true):  admin:org (full)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>Resource names you will see</t>
         </is>
       </c>
     </row>
@@ -688,56 +701,66 @@
       <c r="A32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>Pattern: {service}-{env}-{region-short}-{number}</t>
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Resource names you will see</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>Example with defaults (aksapplz, prod, swedencentral, 1):</t>
-        </is>
-      </c>
+      <c r="A34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Resource group for state:     rg-aksapplz-prod-sc-001</t>
+          <t>Pattern: {service}-{env}-{region-short}-{number}</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Resource group for identity:  rg-aksapplz-prod-sc-identity</t>
+          <t>Example with defaults (aksapplz, prod, swedencentral, 1):</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Resource group for runner:    rg-aksapplz-prod-sc-agents     (only with self-hosted runners)</t>
+          <t xml:space="preserve">  Resource group for state:     rg-aksapplz-prod-sc-001</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  GitHub repository:            aksapplz-prod</t>
+          <t xml:space="preserve">  Resource group for identity:  rg-aksapplz-prod-sc-identity</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  GitHub templates repo:        aksapplz-prod-templates</t>
+          <t xml:space="preserve">  Resource group for runner:    rg-aksapplz-prod-sc-agents     (only with self-hosted runners)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  GitHub repository:            aksapplz-prod</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  GitHub templates repo:        aksapplz-prod-templates</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  Approver team:                aksapplz-prod-approvers</t>
         </is>
@@ -754,7 +777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -763,6 +786,8 @@
     <col width="55" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -775,7 +800,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Fill in the yellow column. Each row matches one question the wizard will ask you.</t>
+          <t>Fill in the yellow columns. Each row matches one question the wizard will ask you. Use 'Reference' for the Microsoft Learn docs and 'Comments' for your own notes.</t>
         </is>
       </c>
     </row>
@@ -808,6 +833,16 @@
       <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Your value</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Comments</t>
         </is>
       </c>
     </row>
@@ -822,6 +857,8 @@
       <c r="D5" s="7" t="n"/>
       <c r="E5" s="7" t="n"/>
       <c r="F5" s="7" t="n"/>
+      <c r="G5" s="7" t="n"/>
+      <c r="H5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
@@ -853,6 +890,12 @@
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr"/>
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
@@ -877,6 +920,12 @@
       </c>
       <c r="E7" s="9" t="inlineStr"/>
       <c r="F7" s="10" t="inlineStr"/>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
@@ -907,6 +956,12 @@
         </is>
       </c>
       <c r="F8" s="10" t="inlineStr"/>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
@@ -937,6 +992,12 @@
         </is>
       </c>
       <c r="F9" s="10" t="inlineStr"/>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr"/>
@@ -949,6 +1010,8 @@
       <c r="D10" s="7" t="n"/>
       <c r="E10" s="7" t="n"/>
       <c r="F10" s="7" t="n"/>
+      <c r="G10" s="7" t="n"/>
+      <c r="H10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
@@ -977,6 +1040,12 @@
         </is>
       </c>
       <c r="F11" s="10" t="inlineStr"/>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
@@ -1006,6 +1075,12 @@
         </is>
       </c>
       <c r="F12" s="10" t="inlineStr"/>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
@@ -1030,6 +1105,12 @@
       </c>
       <c r="E13" s="9" t="inlineStr"/>
       <c r="F13" s="10" t="inlineStr"/>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr"/>
@@ -1042,6 +1123,8 @@
       <c r="D14" s="7" t="n"/>
       <c r="E14" s="7" t="n"/>
       <c r="F14" s="7" t="n"/>
+      <c r="G14" s="7" t="n"/>
+      <c r="H14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
@@ -1066,6 +1149,12 @@
       </c>
       <c r="E15" s="9" t="inlineStr"/>
       <c r="F15" s="10" t="inlineStr"/>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H15" s="10" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
@@ -1094,6 +1183,12 @@
         </is>
       </c>
       <c r="F16" s="10" t="inlineStr"/>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H16" s="10" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr"/>
@@ -1106,6 +1201,8 @@
       <c r="D17" s="7" t="n"/>
       <c r="E17" s="7" t="n"/>
       <c r="F17" s="7" t="n"/>
+      <c r="G17" s="7" t="n"/>
+      <c r="H17" s="7" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
@@ -1134,6 +1231,12 @@
         </is>
       </c>
       <c r="F18" s="10" t="inlineStr"/>
+      <c r="G18" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H18" s="10" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
@@ -1162,6 +1265,12 @@
         </is>
       </c>
       <c r="F19" s="10" t="inlineStr"/>
+      <c r="G19" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H19" s="10" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
@@ -1190,6 +1299,12 @@
         </is>
       </c>
       <c r="F20" s="10" t="inlineStr"/>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H20" s="10" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
@@ -1218,6 +1333,12 @@
         </is>
       </c>
       <c r="F21" s="10" t="inlineStr"/>
+      <c r="G21" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H21" s="10" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr"/>
@@ -1230,6 +1351,8 @@
       <c r="D22" s="7" t="n"/>
       <c r="E22" s="7" t="n"/>
       <c r="F22" s="7" t="n"/>
+      <c r="G22" s="7" t="n"/>
+      <c r="H22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
@@ -1258,6 +1381,12 @@
         </is>
       </c>
       <c r="F23" s="10" t="inlineStr"/>
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H23" s="10" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
@@ -1286,6 +1415,12 @@
         </is>
       </c>
       <c r="F24" s="10" t="inlineStr"/>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H24" s="10" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
@@ -1314,6 +1449,12 @@
         </is>
       </c>
       <c r="F25" s="10" t="inlineStr"/>
+      <c r="G25" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H25" s="10" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
@@ -1342,6 +1483,12 @@
         </is>
       </c>
       <c r="F26" s="10" t="inlineStr"/>
+      <c r="G26" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H26" s="10" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
@@ -1370,6 +1517,12 @@
         </is>
       </c>
       <c r="F27" s="10" t="inlineStr"/>
+      <c r="G27" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H27" s="10" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
@@ -1398,6 +1551,12 @@
         </is>
       </c>
       <c r="F28" s="10" t="inlineStr"/>
+      <c r="G28" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H28" s="10" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
@@ -1426,6 +1585,12 @@
         </is>
       </c>
       <c r="F29" s="10" t="inlineStr"/>
+      <c r="G29" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H29" s="10" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
@@ -1454,6 +1619,12 @@
         </is>
       </c>
       <c r="F30" s="10" t="inlineStr"/>
+      <c r="G30" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H30" s="10" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr"/>
@@ -1466,6 +1637,8 @@
       <c r="D31" s="7" t="n"/>
       <c r="E31" s="7" t="n"/>
       <c r="F31" s="7" t="n"/>
+      <c r="G31" s="7" t="n"/>
+      <c r="H31" s="7" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
@@ -1494,6 +1667,12 @@
         </is>
       </c>
       <c r="F32" s="10" t="inlineStr"/>
+      <c r="G32" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H32" s="10" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
@@ -1522,6 +1701,12 @@
         </is>
       </c>
       <c r="F33" s="10" t="inlineStr"/>
+      <c r="G33" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H33" s="10" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
@@ -1551,6 +1736,12 @@
         </is>
       </c>
       <c r="F34" s="10" t="inlineStr"/>
+      <c r="G34" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H34" s="10" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
@@ -1579,6 +1770,12 @@
         </is>
       </c>
       <c r="F35" s="10" t="inlineStr"/>
+      <c r="G35" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H35" s="10" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr"/>
@@ -1591,6 +1788,8 @@
       <c r="D36" s="7" t="n"/>
       <c r="E36" s="7" t="n"/>
       <c r="F36" s="7" t="n"/>
+      <c r="G36" s="7" t="n"/>
+      <c r="H36" s="7" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
@@ -1619,6 +1818,12 @@
         </is>
       </c>
       <c r="F37" s="10" t="inlineStr"/>
+      <c r="G37" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H37" s="10" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr"/>
@@ -1631,6 +1836,8 @@
       <c r="D38" s="7" t="n"/>
       <c r="E38" s="7" t="n"/>
       <c r="F38" s="7" t="n"/>
+      <c r="G38" s="7" t="n"/>
+      <c r="H38" s="7" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
@@ -1659,6 +1866,12 @@
         </is>
       </c>
       <c r="F39" s="10" t="inlineStr"/>
+      <c r="G39" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H39" s="10" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
@@ -1687,6 +1900,12 @@
         </is>
       </c>
       <c r="F40" s="10" t="inlineStr"/>
+      <c r="G40" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H40" s="10" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
@@ -1715,6 +1934,12 @@
         </is>
       </c>
       <c r="F41" s="10" t="inlineStr"/>
+      <c r="G41" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H41" s="10" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr"/>
@@ -1727,6 +1952,8 @@
       <c r="D42" s="7" t="n"/>
       <c r="E42" s="7" t="n"/>
       <c r="F42" s="7" t="n"/>
+      <c r="G42" s="7" t="n"/>
+      <c r="H42" s="7" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
@@ -1756,6 +1983,12 @@
         </is>
       </c>
       <c r="F43" s="10" t="inlineStr"/>
+      <c r="G43" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H43" s="10" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="8" t="inlineStr">
@@ -1785,6 +2018,12 @@
         </is>
       </c>
       <c r="F44" s="10" t="inlineStr"/>
+      <c r="G44" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H44" s="10" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr"/>
@@ -1797,6 +2036,8 @@
       <c r="D45" s="7" t="n"/>
       <c r="E45" s="7" t="n"/>
       <c r="F45" s="7" t="n"/>
+      <c r="G45" s="7" t="n"/>
+      <c r="H45" s="7" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
@@ -1825,6 +2066,12 @@
         </is>
       </c>
       <c r="F46" s="10" t="inlineStr"/>
+      <c r="G46" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H46" s="10" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
@@ -1853,6 +2100,12 @@
         </is>
       </c>
       <c r="F47" s="10" t="inlineStr"/>
+      <c r="G47" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H47" s="10" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
@@ -1877,6 +2130,12 @@
       </c>
       <c r="E48" s="9" t="inlineStr"/>
       <c r="F48" s="10" t="inlineStr"/>
+      <c r="G48" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H48" s="10" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
@@ -1905,6 +2164,12 @@
         </is>
       </c>
       <c r="F49" s="10" t="inlineStr"/>
+      <c r="G49" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H49" s="10" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr"/>
@@ -1917,6 +2182,8 @@
       <c r="D50" s="7" t="n"/>
       <c r="E50" s="7" t="n"/>
       <c r="F50" s="7" t="n"/>
+      <c r="G50" s="7" t="n"/>
+      <c r="H50" s="7" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
@@ -1945,6 +2212,12 @@
         </is>
       </c>
       <c r="F51" s="10" t="inlineStr"/>
+      <c r="G51" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H51" s="10" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
@@ -1973,6 +2246,12 @@
         </is>
       </c>
       <c r="F52" s="10" t="inlineStr"/>
+      <c r="G52" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H52" s="10" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
@@ -2001,6 +2280,12 @@
         </is>
       </c>
       <c r="F53" s="10" t="inlineStr"/>
+      <c r="G53" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H53" s="10" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
@@ -2029,6 +2314,12 @@
         </is>
       </c>
       <c r="F54" s="10" t="inlineStr"/>
+      <c r="G54" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H54" s="10" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
@@ -2057,6 +2348,12 @@
         </is>
       </c>
       <c r="F55" s="10" t="inlineStr"/>
+      <c r="G55" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H55" s="10" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="8" t="inlineStr">
@@ -2085,6 +2382,12 @@
         </is>
       </c>
       <c r="F56" s="10" t="inlineStr"/>
+      <c r="G56" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H56" s="10" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
@@ -2113,6 +2416,12 @@
         </is>
       </c>
       <c r="F57" s="10" t="inlineStr"/>
+      <c r="G57" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H57" s="10" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="8" t="inlineStr">
@@ -2141,6 +2450,12 @@
         </is>
       </c>
       <c r="F58" s="10" t="inlineStr"/>
+      <c r="G58" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H58" s="10" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
@@ -2169,6 +2484,12 @@
         </is>
       </c>
       <c r="F59" s="10" t="inlineStr"/>
+      <c r="G59" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H59" s="10" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
@@ -2197,6 +2518,12 @@
         </is>
       </c>
       <c r="F60" s="10" t="inlineStr"/>
+      <c r="G60" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H60" s="10" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
@@ -2225,6 +2552,12 @@
         </is>
       </c>
       <c r="F61" s="10" t="inlineStr"/>
+      <c r="G61" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H61" s="10" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="8" t="inlineStr">
@@ -2253,6 +2586,12 @@
         </is>
       </c>
       <c r="F62" s="10" t="inlineStr"/>
+      <c r="G62" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H62" s="10" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
@@ -2281,6 +2620,12 @@
         </is>
       </c>
       <c r="F63" s="10" t="inlineStr"/>
+      <c r="G63" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H63" s="10" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="8" t="inlineStr">
@@ -2309,6 +2654,12 @@
         </is>
       </c>
       <c r="F64" s="10" t="inlineStr"/>
+      <c r="G64" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H64" s="10" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
@@ -2337,6 +2688,12 @@
         </is>
       </c>
       <c r="F65" s="10" t="inlineStr"/>
+      <c r="G65" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H65" s="10" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
@@ -2365,22 +2722,28 @@
         </is>
       </c>
       <c r="F66" s="10" t="inlineStr"/>
+      <c r="G66" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H66" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="B38:F38"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B42:F42"/>
-    <mergeCell ref="B5:F5"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="B45:F45"/>
-    <mergeCell ref="B22:F22"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B36:F36"/>
-    <mergeCell ref="B50:F50"/>
-    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="B22:H22"/>
+    <mergeCell ref="B14:H14"/>
+    <mergeCell ref="B36:H36"/>
+    <mergeCell ref="B50:H50"/>
+    <mergeCell ref="B17:H17"/>
+    <mergeCell ref="B42:H42"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="B45:H45"/>
+    <mergeCell ref="B38:H38"/>
+    <mergeCell ref="B10:H10"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="B31:H31"/>
   </mergeCells>
   <dataValidations count="25">
     <dataValidation sqref="F6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -2459,6 +2822,59 @@
       <formula1>"true,false"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="rId51"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2469,7 +2885,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -2477,6 +2893,8 @@
     <col width="45" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -2519,6 +2937,16 @@
           <t>Your value</t>
         </is>
       </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Comments</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -2530,6 +2958,8 @@
       <c r="C5" s="7" t="n"/>
       <c r="D5" s="7" t="n"/>
       <c r="E5" s="7" t="n"/>
+      <c r="F5" s="7" t="n"/>
+      <c r="G5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -2554,6 +2984,12 @@
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr"/>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -2577,6 +3013,12 @@
         </is>
       </c>
       <c r="E7" s="10" t="inlineStr"/>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -2600,6 +3042,12 @@
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr"/>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -2611,6 +3059,8 @@
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="n"/>
       <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -2634,6 +3084,12 @@
         </is>
       </c>
       <c r="E10" s="10" t="inlineStr"/>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -2657,6 +3113,12 @@
         </is>
       </c>
       <c r="E11" s="10" t="inlineStr"/>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -2680,6 +3142,12 @@
         </is>
       </c>
       <c r="E12" s="10" t="inlineStr"/>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -2691,6 +3159,8 @@
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="7" t="n"/>
       <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
@@ -2715,6 +3185,12 @@
         </is>
       </c>
       <c r="E14" s="10" t="inlineStr"/>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
@@ -2738,6 +3214,12 @@
         </is>
       </c>
       <c r="E15" s="10" t="inlineStr"/>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
@@ -2761,6 +3243,12 @@
         </is>
       </c>
       <c r="E16" s="10" t="inlineStr"/>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
@@ -2784,6 +3272,12 @@
         </is>
       </c>
       <c r="E17" s="10" t="inlineStr"/>
+      <c r="F17" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -2795,6 +3289,8 @@
       <c r="C18" s="7" t="n"/>
       <c r="D18" s="7" t="n"/>
       <c r="E18" s="7" t="n"/>
+      <c r="F18" s="7" t="n"/>
+      <c r="G18" s="7" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -2818,6 +3314,12 @@
         </is>
       </c>
       <c r="E19" s="10" t="inlineStr"/>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="G19" s="10" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
@@ -2841,6 +3343,12 @@
         </is>
       </c>
       <c r="E20" s="10" t="inlineStr"/>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -2852,6 +3360,8 @@
       <c r="C21" s="7" t="n"/>
       <c r="D21" s="7" t="n"/>
       <c r="E21" s="7" t="n"/>
+      <c r="F21" s="7" t="n"/>
+      <c r="G21" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
@@ -2875,6 +3385,12 @@
         </is>
       </c>
       <c r="E22" s="10" t="inlineStr"/>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="G22" s="10" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
@@ -2898,6 +3414,12 @@
         </is>
       </c>
       <c r="E23" s="10" t="inlineStr"/>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
@@ -2921,6 +3443,12 @@
         </is>
       </c>
       <c r="E24" s="10" t="inlineStr"/>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="G24" s="10" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -2932,6 +3460,8 @@
       <c r="C25" s="7" t="n"/>
       <c r="D25" s="7" t="n"/>
       <c r="E25" s="7" t="n"/>
+      <c r="F25" s="7" t="n"/>
+      <c r="G25" s="7" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
@@ -2955,17 +3485,23 @@
         </is>
       </c>
       <c r="E26" s="10" t="inlineStr"/>
+      <c r="F26" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="G26" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A21:E21"/>
-    <mergeCell ref="A18:E18"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A25:E25"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A13:E13"/>
-    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="A5:G5"/>
   </mergeCells>
   <dataValidations count="4">
     <dataValidation sqref="E14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -2981,6 +3517,24 @@
       <formula1>"WAF_v2,Standard_v2"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId16"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(grafana): private by default via private endpoint (WAF/CAF) [v1.15.0]
</commit_message>
<xml_diff>
--- a/config/checklist.xlsx
+++ b/config/checklist.xlsx
@@ -777,7 +777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2392,17 +2392,17 @@
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t>11f</t>
+          <t>11e2</t>
         </is>
       </c>
       <c r="B57" s="9" t="inlineStr">
         <is>
-          <t>enable_app_gateway</t>
+          <t>grafana_public_access</t>
         </is>
       </c>
       <c r="C57" s="9" t="inlineStr">
         <is>
-          <t>Application Gateway with a Web Application Firewall in front of the cluster.</t>
+          <t>Public network access to Managed Grafana. Recommended false (private via private endpoint); a Grafana private endpoint + private DNS zone are created automatically when private endpoints are enabled.</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="F57" s="10" t="inlineStr"/>
@@ -2426,27 +2426,27 @@
     <row r="58">
       <c r="A58" s="8" t="inlineStr">
         <is>
-          <t>11f2</t>
+          <t>11f</t>
         </is>
       </c>
       <c r="B58" s="9" t="inlineStr">
         <is>
-          <t>ingress_controller</t>
+          <t>enable_app_gateway</t>
         </is>
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
-          <t>Only used when enable_app_gateway (11f) is true. Application Gateway acts as a reverse proxy in front of an INTERNAL in-cluster ingress controller: istio (managed Istio internal gateway — auto-selected when Istio 11j is on), traefik (deployed internally for you), or manual (you deploy your own). nginx is not offered (ingress-nginx is being retired). The CD pipeline auto-wires the controller's private IP into the gateway backend pool.</t>
+          <t>Application Gateway with a Web Application Firewall in front of the cluster.</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>istio | traefik | manual</t>
+          <t>true | false</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>traefik  (istio when enable_istio is true)</t>
+          <t>true</t>
         </is>
       </c>
       <c r="F58" s="10" t="inlineStr"/>
@@ -2460,27 +2460,27 @@
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>11f3</t>
+          <t>11f2</t>
         </is>
       </c>
       <c r="B59" s="9" t="inlineStr">
         <is>
-          <t>appgw_tls_key_vault_secret_id</t>
+          <t>ingress_controller</t>
         </is>
       </c>
       <c r="C59" s="9" t="inlineStr">
         <is>
-          <t>Optional. Key Vault secret ID of the TLS certificate for the Application Gateway HTTPS:443 listener (also adds an HTTP→HTTPS redirect). The gateway reads it with the AKS identity. Leave blank to serve HTTP:80 only; you can add TLS later.</t>
+          <t>Only used when enable_app_gateway (11f) is true. Application Gateway acts as a reverse proxy in front of an INTERNAL in-cluster ingress controller: istio (managed Istio internal gateway — auto-selected when Istio 11j is on), traefik (deployed internally for you), or manual (you deploy your own). nginx is not offered (ingress-nginx is being retired). The CD pipeline auto-wires the controller's private IP into the gateway backend pool.</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Key Vault secret URI, or blank</t>
+          <t>istio | traefik | manual</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>(blank = HTTP:80 only)</t>
+          <t>traefik  (istio when enable_istio is true)</t>
         </is>
       </c>
       <c r="F59" s="10" t="inlineStr"/>
@@ -2494,27 +2494,27 @@
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
         <is>
-          <t>11p</t>
+          <t>11f3</t>
         </is>
       </c>
       <c r="B60" s="9" t="inlineStr">
         <is>
-          <t>enable_agc</t>
+          <t>appgw_tls_key_vault_secret_id</t>
         </is>
       </c>
       <c r="C60" s="9" t="inlineStr">
         <is>
-          <t>Application Gateway for Containers (ALB). Provisions a delegated subnet (5h) + NSG; the in-cluster ALB Controller manages the gateway. Coexists with enable_app_gateway.</t>
+          <t>Optional. Key Vault secret ID of the TLS certificate for the Application Gateway HTTPS:443 listener (also adds an HTTP→HTTPS redirect). The gateway reads it with the AKS identity. Leave blank to serve HTTP:80 only; you can add TLS later.</t>
         </is>
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>true | false</t>
+          <t>Key Vault secret URI, or blank</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>(blank = HTTP:80 only)</t>
         </is>
       </c>
       <c r="F60" s="10" t="inlineStr"/>
@@ -2528,17 +2528,17 @@
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t>11g</t>
+          <t>11p</t>
         </is>
       </c>
       <c r="B61" s="9" t="inlineStr">
         <is>
-          <t>enable_keda</t>
+          <t>enable_agc</t>
         </is>
       </c>
       <c r="C61" s="9" t="inlineStr">
         <is>
-          <t>Auto-scales pods based on events (queue length, HTTP requests, etc.).</t>
+          <t>Application Gateway for Containers (ALB). Provisions a delegated subnet (5h) + NSG; the in-cluster ALB Controller manages the gateway. Coexists with enable_app_gateway.</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
@@ -2548,7 +2548,7 @@
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="F61" s="10" t="inlineStr"/>
@@ -2562,17 +2562,17 @@
     <row r="62">
       <c r="A62" s="8" t="inlineStr">
         <is>
-          <t>11h</t>
+          <t>11g</t>
         </is>
       </c>
       <c r="B62" s="9" t="inlineStr">
         <is>
-          <t>enable_vpa</t>
+          <t>enable_keda</t>
         </is>
       </c>
       <c r="C62" s="9" t="inlineStr">
         <is>
-          <t>Auto-adjusts CPU and memory requests for pods.</t>
+          <t>Auto-scales pods based on events (queue length, HTTP requests, etc.).</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
@@ -2582,7 +2582,7 @@
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>false  (true for regulated / multi-region)</t>
+          <t>true</t>
         </is>
       </c>
       <c r="F62" s="10" t="inlineStr"/>
@@ -2596,17 +2596,17 @@
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t>11i</t>
+          <t>11h</t>
         </is>
       </c>
       <c r="B63" s="9" t="inlineStr">
         <is>
-          <t>enable_node_auto_provisioning</t>
+          <t>enable_vpa</t>
         </is>
       </c>
       <c r="C63" s="9" t="inlineStr">
         <is>
-          <t>Cluster creates new node sizes on demand instead of using fixed pools.</t>
+          <t>Auto-adjusts CPU and memory requests for pods.</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
@@ -2616,7 +2616,7 @@
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>false  (true for multi-region)</t>
+          <t>false  (true for regulated / multi-region)</t>
         </is>
       </c>
       <c r="F63" s="10" t="inlineStr"/>
@@ -2630,17 +2630,17 @@
     <row r="64">
       <c r="A64" s="8" t="inlineStr">
         <is>
-          <t>11j</t>
+          <t>11i</t>
         </is>
       </c>
       <c r="B64" s="9" t="inlineStr">
         <is>
-          <t>enable_istio</t>
+          <t>enable_node_auto_provisioning</t>
         </is>
       </c>
       <c r="C64" s="9" t="inlineStr">
         <is>
-          <t>Service mesh with mTLS between pods. Needed for some compliance standards.</t>
+          <t>Cluster creates new node sizes on demand instead of using fixed pools.</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
@@ -2650,7 +2650,7 @@
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>false  (true for regulated)</t>
+          <t>false  (true for multi-region)</t>
         </is>
       </c>
       <c r="F64" s="10" t="inlineStr"/>
@@ -2664,17 +2664,17 @@
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t>11k</t>
+          <t>11j</t>
         </is>
       </c>
       <c r="B65" s="9" t="inlineStr">
         <is>
-          <t>enable_flux</t>
+          <t>enable_istio</t>
         </is>
       </c>
       <c r="C65" s="9" t="inlineStr">
         <is>
-          <t>GitOps — the cluster pulls its configuration from a Git repo.</t>
+          <t>Service mesh with mTLS between pods. Needed for some compliance standards.</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
@@ -2684,7 +2684,7 @@
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>false  (true for multi-region)</t>
+          <t>false  (true for regulated)</t>
         </is>
       </c>
       <c r="F65" s="10" t="inlineStr"/>
@@ -2698,17 +2698,17 @@
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
         <is>
-          <t>11l</t>
+          <t>11k</t>
         </is>
       </c>
       <c r="B66" s="9" t="inlineStr">
         <is>
-          <t>enable_dapr</t>
+          <t>enable_flux</t>
         </is>
       </c>
       <c r="C66" s="9" t="inlineStr">
         <is>
-          <t>Building blocks for microservices (pub/sub, state, secrets).</t>
+          <t>GitOps — the cluster pulls its configuration from a Git repo.</t>
         </is>
       </c>
       <c r="D66" s="9" t="inlineStr">
@@ -2718,7 +2718,7 @@
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>false  (true for multi-region)</t>
         </is>
       </c>
       <c r="F66" s="10" t="inlineStr"/>
@@ -2732,17 +2732,17 @@
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
         <is>
-          <t>11m</t>
+          <t>11l</t>
         </is>
       </c>
       <c r="B67" s="9" t="inlineStr">
         <is>
-          <t>enable_fips</t>
+          <t>enable_dapr</t>
         </is>
       </c>
       <c r="C67" s="9" t="inlineStr">
         <is>
-          <t>Use FIPS 140-2 compliant node OS (US Federal / PCI).</t>
+          <t>Building blocks for microservices (pub/sub, state, secrets).</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
@@ -2752,7 +2752,7 @@
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>false  (true for regulated)</t>
+          <t>false</t>
         </is>
       </c>
       <c r="F67" s="10" t="inlineStr"/>
@@ -2766,17 +2766,17 @@
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
         <is>
-          <t>11n</t>
+          <t>11m</t>
         </is>
       </c>
       <c r="B68" s="9" t="inlineStr">
         <is>
-          <t>enable_backup</t>
+          <t>enable_fips</t>
         </is>
       </c>
       <c r="C68" s="9" t="inlineStr">
         <is>
-          <t>Azure Backup for cluster resources and persistent volumes.</t>
+          <t>Use FIPS 140-2 compliant node OS (US Federal / PCI).</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
@@ -2786,7 +2786,7 @@
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>false  (true for regulated / multi-region)</t>
+          <t>false  (true for regulated)</t>
         </is>
       </c>
       <c r="F68" s="10" t="inlineStr"/>
@@ -2800,17 +2800,17 @@
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
         <is>
-          <t>11o</t>
+          <t>11n</t>
         </is>
       </c>
       <c r="B69" s="9" t="inlineStr">
         <is>
-          <t>enable_cost_analysis</t>
+          <t>enable_backup</t>
         </is>
       </c>
       <c r="C69" s="9" t="inlineStr">
         <is>
-          <t>Cost breakdown per namespace in the Azure portal.</t>
+          <t>Azure Backup for cluster resources and persistent volumes.</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
@@ -2820,7 +2820,7 @@
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>false  (true for regulated)</t>
+          <t>false  (true for regulated / multi-region)</t>
         </is>
       </c>
       <c r="F69" s="10" t="inlineStr"/>
@@ -2830,6 +2830,40 @@
         </is>
       </c>
       <c r="H69" s="10" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="8" t="inlineStr">
+        <is>
+          <t>11o</t>
+        </is>
+      </c>
+      <c r="B70" s="9" t="inlineStr">
+        <is>
+          <t>enable_cost_analysis</t>
+        </is>
+      </c>
+      <c r="C70" s="9" t="inlineStr">
+        <is>
+          <t>Cost breakdown per namespace in the Azure portal.</t>
+        </is>
+      </c>
+      <c r="D70" s="9" t="inlineStr">
+        <is>
+          <t>true | false</t>
+        </is>
+      </c>
+      <c r="E70" s="9" t="inlineStr">
+        <is>
+          <t>false  (true for regulated)</t>
+        </is>
+      </c>
+      <c r="F70" s="10" t="inlineStr"/>
+      <c r="G70" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H70" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -2847,7 +2881,7 @@
     <mergeCell ref="B5:H5"/>
     <mergeCell ref="B31:H31"/>
   </mergeCells>
-  <dataValidations count="27">
+  <dataValidations count="28">
     <dataValidation sqref="F6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"single_region_baseline,multi_region_baseline,single_region_regulated,multi_region_regulated"</formula1>
     </dataValidation>
@@ -2897,10 +2931,10 @@
       <formula1>"true,false"</formula1>
     </dataValidation>
     <dataValidation sqref="F58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"true,false"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"istio,traefik,manual"</formula1>
-    </dataValidation>
-    <dataValidation sqref="F60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"true,false"</formula1>
     </dataValidation>
     <dataValidation sqref="F61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"true,false"</formula1>
@@ -2927,6 +2961,9 @@
       <formula1>"true,false"</formula1>
     </dataValidation>
     <dataValidation sqref="F69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"true,false"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F70" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"true,false"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2985,6 +3022,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="rId55"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(autoscaler): expose opt-in cluster autoscaler profile (v1.17.0)
Add a null-defaulting auto_scaler_profile object variable plumbed root ->
region module -> AVM auto_scaler_profile across all three terraform trees.
Defaults keep native AKS behaviour (no change to existing deployments).

Rather than shipping an opinionated cluster-wide profile, expose and explain
it: new Advanced > Cluster autoscaler tuning docs page (trade-off, AKS
defaults, Microsoft example cost/performance profiles, tfvars snippets),
configuration reference row, day-2 runbook cross-link, and an optional
awareness row in the planning checklist. expander is plan-time validated.

Closes #13
</commit_message>
<xml_diff>
--- a/config/checklist.xlsx
+++ b/config/checklist.xlsx
@@ -777,7 +777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H70"/>
+  <dimension ref="A1:H71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2470,17 +2470,17 @@
       </c>
       <c r="C59" s="9" t="inlineStr">
         <is>
-          <t>Only used when enable_app_gateway (11f) is true. Application Gateway acts as a reverse proxy in front of an INTERNAL in-cluster ingress controller: istio (managed Istio internal gateway — auto-selected when Istio 11j is on), traefik (deployed internally for you), or manual (you deploy your own). nginx is not offered (ingress-nginx is being retired). The CD pipeline auto-wires the controller's private IP into the gateway backend pool.</t>
+          <t>Only used when enable_app_gateway (11f) is true. Application Gateway acts as a reverse proxy in front of an INTERNAL in-cluster ingress controller: istio (managed Istio internal gateway — set up and auto-wired for you; auto-selected when Istio 11j is on) or manual (baseline only — you install and wire your own open-source ingress controller). Only istio is wired by the CD pipeline; manual leaves the ingress controller and backend-pool wiring to you.</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>istio | traefik | manual</t>
+          <t>istio | manual</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>traefik  (istio when enable_istio is true)</t>
+          <t>manual  (istio when enable_istio is true)</t>
         </is>
       </c>
       <c r="F59" s="10" t="inlineStr"/>
@@ -2864,6 +2864,40 @@
         </is>
       </c>
       <c r="H70" s="10" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="8" t="inlineStr">
+        <is>
+          <t>11p</t>
+        </is>
+      </c>
+      <c r="B71" s="9" t="inlineStr">
+        <is>
+          <t>auto_scaler_profile</t>
+        </is>
+      </c>
+      <c r="C71" s="9" t="inlineStr">
+        <is>
+          <t>Day-2 (optional): fine-tune the cluster autoscaler for cost vs performance. Keep AKS defaults unless Azure Advisor flags idle nodes. See docs.</t>
+        </is>
+      </c>
+      <c r="D71" s="9" t="inlineStr">
+        <is>
+          <t>Keep AKS defaults | tune in tfvars</t>
+        </is>
+      </c>
+      <c r="E71" s="9" t="inlineStr">
+        <is>
+          <t>Keep AKS defaults</t>
+        </is>
+      </c>
+      <c r="F71" s="10" t="inlineStr"/>
+      <c r="G71" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H71" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -2934,7 +2968,7 @@
       <formula1>"true,false"</formula1>
     </dataValidation>
     <dataValidation sqref="F59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"istio,traefik,manual"</formula1>
+      <formula1>"istio,manual"</formula1>
     </dataValidation>
     <dataValidation sqref="F61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"true,false"</formula1>
@@ -3023,6 +3057,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="rId56"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: enforce HTTPS/TLS at Application Gateway edge (#21)
Add appgw_tls_mode (keyvault|self_signed|disabled) with keyvault recommended for production, self-signed cert generated inside Key Vault for dev/test, min TLS 1.2 ssl_policy, appgw_https_only toggle, and a breaking production guardrail requiring a customer-provided certificate. Surface the choice in the interactive wizard and the decision checklist. Mirror across terraform/ and ALZ.AKS/templates/terraform/. Keys never stored in repo or state; .gitignore blocks cert formats.
</commit_message>
<xml_diff>
--- a/config/checklist.xlsx
+++ b/config/checklist.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="How to use" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Bootstrap Decisions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Advanced Cluster Settings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bootstrap Decisions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Advanced Cluster Settings" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -777,7 +777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H71"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2494,27 +2494,27 @@
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
         <is>
-          <t>11f3</t>
+          <t>11f2b</t>
         </is>
       </c>
       <c r="B60" s="9" t="inlineStr">
         <is>
-          <t>appgw_tls_key_vault_secret_id</t>
+          <t>appgw_tls_mode</t>
         </is>
       </c>
       <c r="C60" s="9" t="inlineStr">
         <is>
-          <t>Optional. Key Vault secret ID of the TLS certificate for the Application Gateway HTTPS:443 listener (also adds an HTTP→HTTPS redirect). The gateway reads it with the AKS identity. Leave blank to serve HTTP:80 only; you can add TLS later.</t>
+          <t>How the Application Gateway terminates TLS at the internet edge. 'keyvault' = you bring your own certificate (RECOMMENDED for production; a customer-owned certificate must be used in production per Microsoft guidance and PCI-DSS). 'self_signed' = the accelerator generates a certificate inside Key Vault (the private key never leaves Key Vault and is never stored in the repo or state) — DEV/TEST only and blocked for production environments. 'disabled' = HTTP:80 only, no TLS. TLS 1.2 is always the minimum whenever TLS is on. Setting appgw_tls_key_vault_secret_id (11f3) automatically forces 'keyvault'.</t>
         </is>
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>Key Vault secret URI, or blank</t>
+          <t>keyvault | self_signed | disabled</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>(blank = HTTP:80 only)</t>
+          <t>self_signed  (keyvault required for production)</t>
         </is>
       </c>
       <c r="F60" s="10" t="inlineStr"/>
@@ -2528,27 +2528,27 @@
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t>11p</t>
+          <t>11f3</t>
         </is>
       </c>
       <c r="B61" s="9" t="inlineStr">
         <is>
-          <t>enable_agc</t>
+          <t>appgw_tls_key_vault_secret_id</t>
         </is>
       </c>
       <c r="C61" s="9" t="inlineStr">
         <is>
-          <t>Application Gateway for Containers (ALB). Provisions a delegated subnet (5h) + NSG; the in-cluster ALB Controller manages the gateway. Coexists with enable_app_gateway.</t>
+          <t>Customer-provided TLS certificate for the HTTPS:443 listener — used when appgw_tls_mode (11f2b) is 'keyvault'. Provide the Key Vault secret ID (URL) only; the certificate and its private key are never stored in the repo or Terraform state, and the gateway reads the cert with the AKS identity over the private endpoint. Setting this automatically selects 'keyvault' mode. Leave blank for self_signed / disabled.</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>true | false</t>
+          <t>Key Vault secret URI, or blank</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>(blank; required for production)</t>
         </is>
       </c>
       <c r="F61" s="10" t="inlineStr"/>
@@ -2562,17 +2562,17 @@
     <row r="62">
       <c r="A62" s="8" t="inlineStr">
         <is>
-          <t>11g</t>
+          <t>11f4</t>
         </is>
       </c>
       <c r="B62" s="9" t="inlineStr">
         <is>
-          <t>enable_keda</t>
+          <t>appgw_https_only</t>
         </is>
       </c>
       <c r="C62" s="9" t="inlineStr">
         <is>
-          <t>Auto-scales pods based on events (queue length, HTTP requests, etc.).</t>
+          <t>Serve HTTPS only and drop the HTTP:80 listener (no HTTP→HTTPS redirect). Only used when TLS is on (11f2b keyvault or self_signed). Default false keeps HTTP:80 redirecting to HTTPS:443.</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
@@ -2582,7 +2582,7 @@
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="F62" s="10" t="inlineStr"/>
@@ -2596,17 +2596,17 @@
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t>11h</t>
+          <t>11p</t>
         </is>
       </c>
       <c r="B63" s="9" t="inlineStr">
         <is>
-          <t>enable_vpa</t>
+          <t>enable_agc</t>
         </is>
       </c>
       <c r="C63" s="9" t="inlineStr">
         <is>
-          <t>Auto-adjusts CPU and memory requests for pods.</t>
+          <t>Application Gateway for Containers (ALB). Provisions a delegated subnet (5h) + NSG; the in-cluster ALB Controller manages the gateway. Coexists with enable_app_gateway.</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
@@ -2616,7 +2616,7 @@
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>false  (true for regulated / multi-region)</t>
+          <t>false</t>
         </is>
       </c>
       <c r="F63" s="10" t="inlineStr"/>
@@ -2630,17 +2630,17 @@
     <row r="64">
       <c r="A64" s="8" t="inlineStr">
         <is>
-          <t>11i</t>
+          <t>11g</t>
         </is>
       </c>
       <c r="B64" s="9" t="inlineStr">
         <is>
-          <t>enable_node_auto_provisioning</t>
+          <t>enable_keda</t>
         </is>
       </c>
       <c r="C64" s="9" t="inlineStr">
         <is>
-          <t>Cluster creates new node sizes on demand instead of using fixed pools.</t>
+          <t>Auto-scales pods based on events (queue length, HTTP requests, etc.).</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
@@ -2650,7 +2650,7 @@
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>false  (true for multi-region)</t>
+          <t>true</t>
         </is>
       </c>
       <c r="F64" s="10" t="inlineStr"/>
@@ -2664,17 +2664,17 @@
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t>11j</t>
+          <t>11h</t>
         </is>
       </c>
       <c r="B65" s="9" t="inlineStr">
         <is>
-          <t>enable_istio</t>
+          <t>enable_vpa</t>
         </is>
       </c>
       <c r="C65" s="9" t="inlineStr">
         <is>
-          <t>Service mesh with mTLS between pods. Needed for some compliance standards.</t>
+          <t>Auto-adjusts CPU and memory requests for pods.</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
@@ -2684,7 +2684,7 @@
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>false  (true for regulated)</t>
+          <t>false  (true for regulated / multi-region)</t>
         </is>
       </c>
       <c r="F65" s="10" t="inlineStr"/>
@@ -2698,17 +2698,17 @@
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
         <is>
-          <t>11k</t>
+          <t>11i</t>
         </is>
       </c>
       <c r="B66" s="9" t="inlineStr">
         <is>
-          <t>enable_flux</t>
+          <t>enable_node_auto_provisioning</t>
         </is>
       </c>
       <c r="C66" s="9" t="inlineStr">
         <is>
-          <t>GitOps — the cluster pulls its configuration from a Git repo.</t>
+          <t>Cluster creates new node sizes on demand instead of using fixed pools.</t>
         </is>
       </c>
       <c r="D66" s="9" t="inlineStr">
@@ -2732,17 +2732,17 @@
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
         <is>
-          <t>11l</t>
+          <t>11j</t>
         </is>
       </c>
       <c r="B67" s="9" t="inlineStr">
         <is>
-          <t>enable_dapr</t>
+          <t>enable_istio</t>
         </is>
       </c>
       <c r="C67" s="9" t="inlineStr">
         <is>
-          <t>Building blocks for microservices (pub/sub, state, secrets).</t>
+          <t>Service mesh with mTLS between pods. Needed for some compliance standards.</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
@@ -2752,7 +2752,7 @@
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>false  (true for regulated)</t>
         </is>
       </c>
       <c r="F67" s="10" t="inlineStr"/>
@@ -2766,17 +2766,17 @@
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
         <is>
-          <t>11m</t>
+          <t>11k</t>
         </is>
       </c>
       <c r="B68" s="9" t="inlineStr">
         <is>
-          <t>enable_fips</t>
+          <t>enable_flux</t>
         </is>
       </c>
       <c r="C68" s="9" t="inlineStr">
         <is>
-          <t>Use FIPS 140-2 compliant node OS (US Federal / PCI).</t>
+          <t>GitOps — the cluster pulls its configuration from a Git repo.</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
@@ -2786,7 +2786,7 @@
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>false  (true for regulated)</t>
+          <t>false  (true for multi-region)</t>
         </is>
       </c>
       <c r="F68" s="10" t="inlineStr"/>
@@ -2800,17 +2800,17 @@
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
         <is>
-          <t>11n</t>
+          <t>11l</t>
         </is>
       </c>
       <c r="B69" s="9" t="inlineStr">
         <is>
-          <t>enable_backup</t>
+          <t>enable_dapr</t>
         </is>
       </c>
       <c r="C69" s="9" t="inlineStr">
         <is>
-          <t>Azure Backup for cluster resources and persistent volumes.</t>
+          <t>Building blocks for microservices (pub/sub, state, secrets).</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
@@ -2820,7 +2820,7 @@
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>false  (true for regulated / multi-region)</t>
+          <t>false</t>
         </is>
       </c>
       <c r="F69" s="10" t="inlineStr"/>
@@ -2834,17 +2834,17 @@
     <row r="70">
       <c r="A70" s="8" t="inlineStr">
         <is>
-          <t>11o</t>
+          <t>11m</t>
         </is>
       </c>
       <c r="B70" s="9" t="inlineStr">
         <is>
-          <t>enable_cost_analysis</t>
+          <t>enable_fips</t>
         </is>
       </c>
       <c r="C70" s="9" t="inlineStr">
         <is>
-          <t>Cost breakdown per namespace in the Azure portal.</t>
+          <t>Use FIPS 140-2 compliant node OS (US Federal / PCI).</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
@@ -2868,27 +2868,27 @@
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
         <is>
-          <t>11p</t>
+          <t>11n</t>
         </is>
       </c>
       <c r="B71" s="9" t="inlineStr">
         <is>
-          <t>auto_scaler_profile</t>
+          <t>enable_backup</t>
         </is>
       </c>
       <c r="C71" s="9" t="inlineStr">
         <is>
-          <t>Day-2 (optional): fine-tune the cluster autoscaler for cost vs performance. Keep AKS defaults unless Azure Advisor flags idle nodes. See docs.</t>
+          <t>Azure Backup for cluster resources and persistent volumes.</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>Keep AKS defaults | tune in tfvars</t>
+          <t>true | false</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>Keep AKS defaults</t>
+          <t>false  (true for regulated / multi-region)</t>
         </is>
       </c>
       <c r="F71" s="10" t="inlineStr"/>
@@ -2898,6 +2898,176 @@
         </is>
       </c>
       <c r="H71" s="10" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="8" t="inlineStr">
+        <is>
+          <t>11o</t>
+        </is>
+      </c>
+      <c r="B72" s="9" t="inlineStr">
+        <is>
+          <t>enable_cost_analysis</t>
+        </is>
+      </c>
+      <c r="C72" s="9" t="inlineStr">
+        <is>
+          <t>Cost breakdown per namespace in the Azure portal.</t>
+        </is>
+      </c>
+      <c r="D72" s="9" t="inlineStr">
+        <is>
+          <t>true | false</t>
+        </is>
+      </c>
+      <c r="E72" s="9" t="inlineStr">
+        <is>
+          <t>false  (true for regulated)</t>
+        </is>
+      </c>
+      <c r="F72" s="10" t="inlineStr"/>
+      <c r="G72" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H72" s="10" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="8" t="inlineStr">
+        <is>
+          <t>11q</t>
+        </is>
+      </c>
+      <c r="B73" s="9" t="inlineStr">
+        <is>
+          <t>enable_management_jumpbox</t>
+        </is>
+      </c>
+      <c r="C73" s="9" t="inlineStr">
+        <is>
+          <t>Opt-in Azure Bastion + hardened no-public-IP jumpbox VM for private-cluster access (standalone only; ALZ hubs provide Bastion/VPN).</t>
+        </is>
+      </c>
+      <c r="D73" s="9" t="inlineStr">
+        <is>
+          <t>true | false</t>
+        </is>
+      </c>
+      <c r="E73" s="9" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F73" s="10" t="inlineStr"/>
+      <c r="G73" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H73" s="10" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="8" t="inlineStr">
+        <is>
+          <t>11r</t>
+        </is>
+      </c>
+      <c r="B74" s="9" t="inlineStr">
+        <is>
+          <t>jumpbox_vm_size</t>
+        </is>
+      </c>
+      <c r="C74" s="9" t="inlineStr">
+        <is>
+          <t>VM size for the management jumpbox (any valid Azure VM size). Applies only when enable_management_jumpbox = true.</t>
+        </is>
+      </c>
+      <c r="D74" s="9" t="inlineStr">
+        <is>
+          <t>Standard_B2s_v2 | Standard_D2s_v5 | any Azure VM size</t>
+        </is>
+      </c>
+      <c r="E74" s="9" t="inlineStr">
+        <is>
+          <t>Standard_B2s_v2</t>
+        </is>
+      </c>
+      <c r="F74" s="10" t="inlineStr"/>
+      <c r="G74" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H74" s="10" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="8" t="inlineStr">
+        <is>
+          <t>11s</t>
+        </is>
+      </c>
+      <c r="B75" s="9" t="inlineStr">
+        <is>
+          <t>bastion_sku</t>
+        </is>
+      </c>
+      <c r="C75" s="9" t="inlineStr">
+        <is>
+          <t>Azure Bastion SKU for jumpbox access. Standard enables native-client SSH/tunneling; Basic is browser-only. Applies only when enable_management_jumpbox = true.</t>
+        </is>
+      </c>
+      <c r="D75" s="9" t="inlineStr">
+        <is>
+          <t>Standard | Basic</t>
+        </is>
+      </c>
+      <c r="E75" s="9" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="F75" s="10" t="inlineStr"/>
+      <c r="G75" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H75" s="10" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="8" t="inlineStr">
+        <is>
+          <t>11p</t>
+        </is>
+      </c>
+      <c r="B76" s="9" t="inlineStr">
+        <is>
+          <t>auto_scaler_profile</t>
+        </is>
+      </c>
+      <c r="C76" s="9" t="inlineStr">
+        <is>
+          <t>Day-2 (optional): fine-tune the cluster autoscaler for cost vs performance. Keep AKS defaults unless Azure Advisor flags idle nodes. See docs.</t>
+        </is>
+      </c>
+      <c r="D76" s="9" t="inlineStr">
+        <is>
+          <t>Keep AKS defaults | tune in tfvars</t>
+        </is>
+      </c>
+      <c r="E76" s="9" t="inlineStr">
+        <is>
+          <t>Keep AKS defaults</t>
+        </is>
+      </c>
+      <c r="F76" s="10" t="inlineStr"/>
+      <c r="G76" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Learn ↗</t>
+        </is>
+      </c>
+      <c r="H76" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -2915,7 +3085,7 @@
     <mergeCell ref="B5:H5"/>
     <mergeCell ref="B31:H31"/>
   </mergeCells>
-  <dataValidations count="28">
+  <dataValidations count="31">
     <dataValidation sqref="F6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"single_region_baseline,multi_region_baseline,single_region_regulated,multi_region_regulated"</formula1>
     </dataValidation>
@@ -2970,8 +3140,8 @@
     <dataValidation sqref="F59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"istio,manual"</formula1>
     </dataValidation>
-    <dataValidation sqref="F61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"true,false"</formula1>
+    <dataValidation sqref="F60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"keyvault,self_signed,disabled"</formula1>
     </dataValidation>
     <dataValidation sqref="F62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"true,false"</formula1>
@@ -2998,6 +3168,15 @@
       <formula1>"true,false"</formula1>
     </dataValidation>
     <dataValidation sqref="F70" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"true,false"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F71" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"true,false"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"true,false"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F73" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"true,false"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3058,6 +3237,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G73" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G74" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId61"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>